<commit_message>
add stakeholder needs analysis and update glossary
</commit_message>
<xml_diff>
--- a/src/ONR_GLS.xlsx
+++ b/src/ONR_GLS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dar/Documents/bsa-barbershop-case-study/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AF3D76C-492A-E54F-B4EB-C7274C206D5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{357A5AB7-C386-E44C-A484-DA739F3916D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{B525281D-720F-9043-BAFC-8DAF48A3C29E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="70">
   <si>
     <t>Код</t>
   </si>
@@ -193,6 +193,36 @@
 тата, создаваемого командой.</t>
   </si>
   <si>
+    <t>Стейкхолдер</t>
+  </si>
+  <si>
+    <t>ГОСТ 51897-2002</t>
+  </si>
+  <si>
+    <t>Заинтересованная сторона, владелец доли</t>
+  </si>
+  <si>
+    <t>Причастная сторона.</t>
+  </si>
+  <si>
+    <t>Бухгалтер</t>
+  </si>
+  <si>
+    <t>(нем. Buchhalter, Buch — книга, Halter — держатель/держатель книги) — специалист по бухгалтерскому учёту, работающий по системе учёта в соответствии с действующим законодательством.</t>
+  </si>
+  <si>
+    <t>Википедия</t>
+  </si>
+  <si>
+    <t>деятельность по предупреждению, обнаружению, пресечению нарушений в области обеспечения санитарно-эпидемиологического благополучия населения в целях охраны здоровья населения и среды обитания человека. Целью санитарно-эпидемиологического надзора является предупреждение возникновения острых инфекционных заболеваний среди населения.</t>
+  </si>
+  <si>
+    <t>Санитарно-эпидемиологический контроль</t>
+  </si>
+  <si>
+    <t>Санэпиднадзор</t>
+  </si>
+  <si>
     <t>ONR_GLS_001</t>
   </si>
   <si>
@@ -221,6 +251,15 @@
   </si>
   <si>
     <t>ONR_GLS_010</t>
+  </si>
+  <si>
+    <t>ONR_GLS_011</t>
+  </si>
+  <si>
+    <t>ONR_GLS_012</t>
+  </si>
+  <si>
+    <t>ONR_GLS_013</t>
   </si>
 </sst>
 </file>
@@ -264,8 +303,8 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -719,10 +758,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D573AB8C-5CE1-A145-BDF1-F108350FAA04}">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.5" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
     <col min="2" max="2" width="19.83203125" customWidth="1"/>
     <col min="3" max="3" width="31.33203125" customWidth="1"/>
     <col min="4" max="4" width="16.1640625" customWidth="1"/>
@@ -760,7 +799,7 @@
     </row>
     <row r="2" spans="1:8" ht="118" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>9</v>
@@ -786,7 +825,7 @@
     </row>
     <row r="3" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>13</v>
@@ -812,7 +851,7 @@
     </row>
     <row r="4" spans="1:8" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>19</v>
@@ -838,7 +877,7 @@
     </row>
     <row r="5" spans="1:8" ht="50" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>17</v>
@@ -864,7 +903,7 @@
     </row>
     <row r="6" spans="1:8" ht="88" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>21</v>
@@ -890,7 +929,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>30</v>
@@ -916,7 +955,7 @@
     </row>
     <row r="8" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>34</v>
@@ -942,7 +981,7 @@
     </row>
     <row r="9" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>38</v>
@@ -968,7 +1007,7 @@
     </row>
     <row r="10" spans="1:8" ht="130" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>42</v>
@@ -994,7 +1033,7 @@
     </row>
     <row r="11" spans="1:8" ht="96" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>43</v>
@@ -1015,6 +1054,84 @@
         <v>3</v>
       </c>
       <c r="H11" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="A12" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="F12" s="4">
+        <v>46227</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="96" x14ac:dyDescent="0.2">
+      <c r="A13" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F13" s="4">
+        <v>46227</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="192" x14ac:dyDescent="0.2">
+      <c r="A14" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F14" s="4">
+        <v>46227</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H14" s="9" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add as-is, to-be and data streams artifacts
</commit_message>
<xml_diff>
--- a/src/ONR_GLS.xlsx
+++ b/src/ONR_GLS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dar/Documents/bsa-barbershop-case-study/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{357A5AB7-C386-E44C-A484-DA739F3916D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3086AFA-5BD5-E742-95BC-AC47849D348B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{B525281D-720F-9043-BAFC-8DAF48A3C29E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="76">
   <si>
     <t>Код</t>
   </si>
@@ -260,6 +260,24 @@
   </si>
   <si>
     <t>ONR_GLS_013</t>
+  </si>
+  <si>
+    <t>ONR_GLS_014</t>
+  </si>
+  <si>
+    <t>Требование</t>
+  </si>
+  <si>
+    <t>это пригодное для практического использования представление потребности или решения</t>
+  </si>
+  <si>
+    <t>ONR_GLS_015</t>
+  </si>
+  <si>
+    <t>Контекстная диаграмма</t>
+  </si>
+  <si>
+    <t>Она отображает, какие потоки информации или управляющие воздействия передаются извне внутрь системы, а какие из системы наружу, и кто их передает. Контекстная диаграмма не показывает, что делается внутри системы, только «черный ящик». А еще она помогает определить границы системы.</t>
   </si>
 </sst>
 </file>
@@ -320,7 +338,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -382,11 +400,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -423,6 +461,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -758,7 +805,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D573AB8C-5CE1-A145-BDF1-F108350FAA04}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -1135,6 +1182,58 @@
         <v>16</v>
       </c>
     </row>
+    <row r="15" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="A15" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="4">
+        <v>46235</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="144" x14ac:dyDescent="0.2">
+      <c r="A16" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="4">
+        <v>46235</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>